<commit_message>
Dossiers d'importation 2026 : achats importation (05001), entrées en stock (10001) et coût de revient par article
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XYis4EzVZMNdoYCxmLrRh4
</commit_message>
<xml_diff>
--- a/REGISTRE_SOUCHES_CHEQUES_2026.xlsx
+++ b/REGISTRE_SOUCHES_CHEQUES_2026.xlsx
@@ -2130,9 +2130,19 @@
       <c r="A45" s="3" t="n">
         <v>2125744</v>
       </c>
-      <c r="B45" s="3" t="inlineStr"/>
-      <c r="C45" s="3" t="inlineStr"/>
-      <c r="D45" s="3" t="n"/>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>23/04/2026</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>CMA CGM ALGERIE (copie du chèque, facture DZIM1984785)</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="n">
+        <v>41855.09</v>
+      </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
           <t>18/05/2026</t>
@@ -2141,17 +2151,27 @@
       <c r="F45" s="4" t="n">
         <v>41855.09</v>
       </c>
-      <c r="G45" s="3" t="n"/>
-      <c r="H45" s="3" t="inlineStr"/>
-      <c r="I45" s="3" t="inlineStr"/>
-      <c r="J45" s="8" t="inlineStr">
-        <is>
-          <t>Débité sans souche : à identifier</t>
+      <c r="G45" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>40100</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>CMA CGM</t>
+        </is>
+      </c>
+      <c r="J45" s="7" t="inlineStr">
+        <is>
+          <t>Comptabilisé (souche)</t>
         </is>
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>Souche absente des photos : passé en 47000</t>
+          <t>CHQ 2125744 CMA CGM</t>
         </is>
       </c>
     </row>
@@ -3022,7 +3042,7 @@
         </is>
       </c>
       <c r="F73" s="11" t="n">
-        <v>5146631.38</v>
+        <v>5104776.29</v>
       </c>
     </row>
     <row r="74">

</xml_diff>

<commit_message>
Assurance L'Algérienne des Assurances (GIG) 2026-2027 : facture et chèque CPA 2125764
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XYis4EzVZMNdoYCxmLrRh4
</commit_message>
<xml_diff>
--- a/REGISTRE_SOUCHES_CHEQUES_2026.xlsx
+++ b/REGISTRE_SOUCHES_CHEQUES_2026.xlsx
@@ -2737,9 +2737,19 @@
       <c r="A62" s="3" t="n">
         <v>2125764</v>
       </c>
-      <c r="B62" s="3" t="inlineStr"/>
-      <c r="C62" s="3" t="inlineStr"/>
-      <c r="D62" s="3" t="n"/>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>05/08/2026</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>L'ALGERIENNE DES ASSURANCES (GIG) — facture A31014/2026/0000018781283</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="n">
+        <v>5147.25</v>
+      </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
           <t>12/08/2026</t>
@@ -2748,17 +2758,27 @@
       <c r="F62" s="4" t="n">
         <v>5147.25</v>
       </c>
-      <c r="G62" s="3" t="n"/>
-      <c r="H62" s="3" t="inlineStr"/>
-      <c r="I62" s="3" t="inlineStr"/>
-      <c r="J62" s="8" t="inlineStr">
-        <is>
-          <t>Débité sans souche : à identifier</t>
+      <c r="G62" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>40130</t>
+        </is>
+      </c>
+      <c r="I62" s="3" t="inlineStr">
+        <is>
+          <t>L'ALGERIENNE DES ASSURANCES</t>
+        </is>
+      </c>
+      <c r="J62" s="7" t="inlineStr">
+        <is>
+          <t>Comptabilisé (souche)</t>
         </is>
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>Souche absente des photos : passé en 47000</t>
+          <t>CHQ 2125764 AGA ASSURANCE</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3062,7 @@
         </is>
       </c>
       <c r="F73" s="11" t="n">
-        <v>5104776.29</v>
+        <v>5099629.04</v>
       </c>
     </row>
     <row r="74">

</xml_diff>